<commit_message>
Add missing dropdowns across all templates, verify comment dimensions
- FMCG: category dropdown D5:D1004 → Reference_Lists!$B$4:$B$43 (40 categories)
- Manufacturing: category dropdown D5:D1004 → Reference_Lists!$B$4:$B$46 (43 categories)
- Retail: category dropdown D5:D1004 → Reference_Lists!$B$4:$B$108 (105 categories)
- Logistics: fuel_surcharge_clause dropdown AH5:AH504 → Reference_Lists!$E$2:$E$4
- All 104 comments across 4 templates resized (VML confirmed 240–380px wide, 114–204px tall)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/MarginCOS_Data_Template_v3.2_FMCG.xlsx
+++ b/public/downloads/MarginCOS_Data_Template_v3.2_FMCG.xlsx
@@ -32014,7 +32014,7 @@
     <mergeCell ref="R1:T1"/>
     <mergeCell ref="K1:N1"/>
   </mergeCells>
-  <dataValidations count="11">
+  <dataValidations count="12">
     <dataValidation sqref="E5:E1004" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Segment" error="Choose: Mass Market, Mid-Range, or Premium." promptTitle="Segment" prompt="Select the price segment for this SKU." type="list">
       <formula1>"Mass Market,Mid-Range,Premium"</formula1>
       <formula2>0</formula2>
@@ -32058,6 +32058,9 @@
     <dataValidation sqref="B5:B1004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Duplicate SKU ID" error="This SKU ID already exists in your upload. Each row must have a unique SKU ID." type="custom">
       <formula1>COUNTIF($B$5:$B$1004,B5)=1</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation sqref="D5:D1004" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Category" error="Please select from the dropdown list." promptTitle="Category" prompt="Select the product category from the Reference_Lists sheet." type="list" errorStyle="warning">
+      <formula1>=Reference_Lists!$B$4:$B$43</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>